<commit_message>
decouple esqlabsR and reportingFramework
</commit_message>
<xml_diff>
--- a/inst/templates/ProjectConfiguration.xlsx
+++ b/inst/templates/ProjectConfiguration.xlsx
@@ -1,26 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="esqlabsR" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="addons" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
   <si>
     <t xml:space="preserve">Property</t>
   </si>
@@ -152,16 +147,52 @@
   </si>
   <si>
     <t xml:space="preserve">Path to the folder where electronic Package is saved</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parameterIdentificationFile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ParameterIdentification.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name of the excel file with parameter identification task definitions. Must be located in the configurationsFolder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dataFile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name of the excel file with experimental data. Must be located in the dataFolder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">esqlabsRVersion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Version of the esqlabsR package used to create this configuration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ospsuiteReportingFrameworkVersion </t>
+  </si>
+  <si>
+    <t xml:space="preserve">reportsFile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Report.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name of the excel file with plot configurations. Must be located in the "configurationsFolder"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reports.xlsx</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -170,27 +201,17 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="0"/>
     </font>
   </fonts>
   <fills count="2">
@@ -202,7 +223,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -210,49 +231,28 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment textRotation="0" horizontal="center" vertical="bottom" indent="0"/>
+      <protection hidden="0" locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-  </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment textRotation="0" horizontal="general" vertical="bottom" indent="0"/>
+      <protection hidden="0" locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment textRotation="0" horizontal="general" vertical="bottom" indent="0" wrapText="1"/>
+      <protection hidden="0" locked="0"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
 </styleSheet>
 </file>
 
@@ -432,19 +432,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="119.86"/>
+    <col min="1" max="1" width="28.57" hidden="false" outlineLevel="0" customWidth="1"/>
+    <col min="2" max="2" width="25.57" hidden="false" outlineLevel="0" customWidth="1"/>
+    <col min="3" max="3" width="119.86" hidden="false" outlineLevel="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -455,167 +455,262 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+    <row r="5" ht="15" customHeight="1">
+      <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+    <row r="10" ht="15" customHeight="1">
+      <c r="A10" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+    <row r="13" ht="15" customHeight="1">
+      <c r="A13" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+    <row r="14" ht="15" customHeight="1">
+      <c r="A14" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+    <row r="15" ht="15" customHeight="1">
+      <c r="A15" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="2" t="s">
         <v>43</v>
       </c>
     </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.7" right="0.7" top="0.597222222222222" bottom="0.597222222222222" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
+  <headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="0" alignWithMargins="0">
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1" ht="13.5" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" ht="34.5" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2"/>
+      <c r="C2"/>
+    </row>
+    <row r="3" ht="13.5" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" ht="13.5" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="0" alignWithMargins="0">
+    <oddHeader>&amp;L&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P&amp;R</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>